<commit_message>
Sync scenario demo with live tracker: linear ramp, Default/Override, Graph tab
- Safety Anchor % was still the old step function; replaced with the same
  linear ramp (Starting % -> Ending % over Ramp Length years, then flat)
  now used in household_portfolio_engine.xlsx.
- Added Default / Override / Effective columns for the five configured
  inputs on The_Refill_Engine, matching the live tracker's layout.
- Added a Graph tab: Simulated Actual Household Wealth vs. the hurdle
  target (P_track) by year, redrawing live as the scenario selector
  changes. Roth conversion tracking was deliberately left out -- it's a
  personal planning detail unrelated to this demo's market-scenario story.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dyD4f3m3cXsViTiCTbG7n
</commit_message>
<xml_diff>
--- a/household_portfolio_scenario_demo.xlsx
+++ b/household_portfolio_scenario_demo.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables_And_Log" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Account_Tracker" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The_Refill_Engine" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graph" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -182,8 +183,8 @@
     <xf numFmtId="10" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -317,6 +318,177 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Simulated Actual Household Wealth vs. Hurdle Target (P_track)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'The_Refill_Engine'!D62</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="44546A"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'The_Refill_Engine'!$A$63:$A$72</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'The_Refill_Engine'!$D$63:$D$72</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'The_Refill_Engine'!F62</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="1F3864"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'The_Refill_Engine'!$A$63:$A$72</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'The_Refill_Engine'!$F$63:$F$72</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="-10"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Household Wealth ($)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="$#,##0" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9360000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -608,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -685,7 +857,7 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HOW THE FOUR TABS WORK TOGETHER</t>
+          <t>HOW THE FIVE TABS WORK TOGETHER</t>
         </is>
       </c>
       <c r="B14" s="2" t="n"/>
@@ -711,228 +883,247 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="83" customHeight="1">
+    <row r="18" ht="128" customHeight="1">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>The_Refill_Engine -- The decision-making tab, plus the scenario selector. The Quarterly Refill Engine table is the headline output. The Annual SRR Hurdle Model below it now also simulates actual household wealth forward year by year under the selected scenario and compares it to the hurdle target, which is what drives GOOD vs. POOR here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+          <t>The_Refill_Engine -- The decision-making tab, plus the scenario selector. A block of configured inputs (Retirement Start Year, Ramp Length, the G Fund target percentages, etc.) each carry a Default, an optional Override, and the resulting Effective value everything else on the tab actually uses. The Quarterly Refill Engine table is the headline output. The Annual SRR Hurdle Model below it simulates actual household wealth forward year by year under the selected scenario and compares it to the hurdle target, which is what drives GOOD vs. POOR here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="53" customHeight="1">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Graph -- A single chart, read-only, pulling straight from The_Refill_Engine's Annual SRR Hurdle Model: Simulated Actual Household Wealth vs. the hurdle target (P_track), by year, for whichever scenario is currently selected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>COLOR LEGEND</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n"/>
-    </row>
-    <row r="21" ht="38" customHeight="1">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="n"/>
+    </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Pale yellow -- an editable input, pre-filled with an illustrative example value.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="38" customHeight="1">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="3" t="inlineStr">
+    <row r="23" ht="38" customHeight="1">
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>White (no fill) -- a formula, or a fixed scenario assumption; please leave it alone.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="23" customHeight="1">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="3" t="inlineStr">
+    <row r="24" ht="23" customHeight="1">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Ice blue -- a computed summary or headline total.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="23" customHeight="1">
-      <c r="A24" s="7" t="n"/>
-      <c r="B24" s="3" t="inlineStr">
+    <row r="25" ht="23" customHeight="1">
+      <c r="A25" s="7" t="n"/>
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Green (Emergency Liquidity Protocol only) -- the TSP G Fund shield is active.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="38" customHeight="1">
-      <c r="A25" s="8" t="n"/>
-      <c r="B25" s="3" t="inlineStr">
+    <row r="26" ht="38" customHeight="1">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Yellow (Emergency Liquidity Protocol only) -- the G Fund is exhausted; drawing from the cash buffer.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="38" customHeight="1">
-      <c r="A26" s="9" t="n"/>
-      <c r="B26" s="3" t="inlineStr">
+    <row r="27" ht="38" customHeight="1">
+      <c r="A27" s="9" t="n"/>
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Red (Emergency Liquidity Protocol only) -- both cash shields are exhausted; the household is in an emergency-liquidation stage.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>GLOSSARY</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="B29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>Term</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>Definition</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="38" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>COLA</t>
-        </is>
-      </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>The federal Cost-of-Living Adjustment, applied annually to Social Security/federal retirement benefits.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="38" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
+          <t>COLA</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>The federal Cost-of-Living Adjustment, applied annually to Social Security/federal retirement benefits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="38" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
           <t>Hurdle Rate</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>The minimum real (inflation-adjusted) growth rate the portfolio needs to clear to be considered "on track" -- COLA layered on a fixed real-growth baseline.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="23" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="33" ht="23" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>W_t / W_q</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Total dollar outflows (withdrawals) for a given year (t) or quarter (q).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="38" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t>P_track</t>
-        </is>
-      </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>The simulated target portfolio value (the hurdle trajectory) that simulated actual wealth is measured against each year.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="38" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
+          <t>P_track</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>The simulated target portfolio value (the hurdle trajectory) that simulated actual wealth is measured against each year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="38" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>One of three hardcoded, hypothetical annual market-return paths -- Bear, Bull, or Choppy -- selected on The_Refill_Engine tab.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="53" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
+    <row r="36" ht="53" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>Simulated Actual Household Wealth</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>This demo's stand-in for real net worth: last year's simulated wealth, grown by the selected scenario's return for the year, less that year's outflows. Compared against P_track to decide GOOD vs. POOR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="38" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
-        <is>
-          <t>SRR</t>
-        </is>
-      </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>Sequence-of-Returns Risk -- the risk that a downturn early in retirement forces permanent sale of depreciated assets.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="38" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
+          <t>SRR</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>Sequence-of-Returns Risk -- the risk that a downturn early in retirement forces permanent sale of depreciated assets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="38" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
           <t>TSP G Fund</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>The federal Thrift Savings Plan's government-securities fund: principal-protected, instantly liquid, and the household's operating cash vault.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="68" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
+    <row r="39" ht="83" customHeight="1">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Safety Anchor</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
-        <is>
-          <t>The G Fund cash buffer this engine tries to maintain. Set as a step function (on The_Refill_Engine): a higher percentage through the SRR "red zone" -- the first several years of retirement -- then a lower one afterward, applied each year to that year's P_track rather than a frozen snapshot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="53" customHeight="1">
-      <c r="A39" s="11" t="inlineStr">
-        <is>
-          <t>Red Zone</t>
-        </is>
-      </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>The first several years of retirement, when a bad sequence of market returns does the most lasting damage to a portfolio. The Safety Anchor holds a higher percentage during this window.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="38" customHeight="1">
+          <t>The G Fund cash buffer this engine tries to maintain. Ramps linearly (on The_Refill_Engine) from a Starting % down to an Ending % over the Ramp Length, then holds flat -- largest during the early years when SRR risk is heavily front-loaded, easing as that window passes. Applied each year to that year's P_track rather than a frozen snapshot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="53" customHeight="1">
       <c r="A40" s="11" t="inlineStr">
         <is>
+          <t>Ramp Length</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>How many years the G Fund target percentage takes to slide from its Starting % to its Ending %, before holding flat. A configured input on The_Refill_Engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="68" customHeight="1">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>Default / Override / Effective</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>The three-column pattern used for every configured input on The_Refill_Engine. Default is the built-in value; Override is blank unless you want to change it; Effective is whichever one is actually in force, and is what every other formula on the tab references.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="38" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
           <t>Conduit</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>A Traditional IRA used as a pass-through for pre-tax rollovers back into the TSP.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="23" customHeight="1">
-      <c r="A41" s="11" t="inlineStr">
+    <row r="43" ht="23" customHeight="1">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>Allocation Mix</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>Each account's share of total household net worth, shown on Account_Tracker.</t>
         </is>
@@ -940,10 +1131,10 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A29:B29"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A28:B28"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A3:B3"/>
@@ -2033,7 +2224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2076,291 +2267,210 @@
         <v/>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="24" t="inlineStr">
-        <is>
-          <t>Retirement Start Year</t>
-        </is>
-      </c>
-      <c r="B4" s="26" t="n">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="24" t="inlineStr">
-        <is>
-          <t>Age at Retirement Start</t>
-        </is>
-      </c>
-      <c r="B5" s="26" t="n">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="24" t="inlineStr">
-        <is>
-          <t>Red Zone Length (Years)</t>
-        </is>
-      </c>
-      <c r="B6" s="26" t="n">
-        <v>10</v>
+    <row r="4"/>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>CONFIGURED INPUTS — DEFAULT / OVERRIDE / EFFECTIVE</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Override (blank = use Default)</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>Effective (used below)</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>Red Zone Target % (elevated, early retirement)</t>
-        </is>
-      </c>
-      <c r="B7" s="27" t="n">
-        <v>0.35</v>
+          <t>Retirement Start Year</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C7" s="26" t="n"/>
+      <c r="D7" s="27">
+        <f>IF(C7="",B7,C7)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>Post-Red-Zone Target % (steady state)</t>
-        </is>
-      </c>
-      <c r="B8" s="27" t="n">
-        <v>0.25</v>
+          <t>Age at Retirement Start</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>63</v>
+      </c>
+      <c r="C8" s="26" t="n"/>
+      <c r="D8" s="27">
+        <f>IF(C8="",B8,C8)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>Current Safety Anchor %</t>
-        </is>
-      </c>
-      <c r="B9" s="23">
-        <f>IF(YEAR(TODAY())-B4&lt;B6,B7,B8)</f>
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Ramp Length (Years)</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="26" t="n"/>
+      <c r="D9" s="27">
+        <f>IF(C9="",B9,C9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Starting G Fund Target % (elevated, early retirement)</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="23">
+        <f>IF(C10="",B10,C10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>Ending G Fund Target % (steady state)</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="23">
+        <f>IF(C11="",B11,C11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>Current G Fund Target % (Today)</t>
+        </is>
+      </c>
+      <c r="B13" s="23">
+        <f>IF(YEAR(TODAY())-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(YEAR(TODAY())-$D$7)/$D$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>Target Safety Anchor Balance (Year 1 Opening)</t>
         </is>
       </c>
-      <c r="B10" s="22">
-        <f>B3*B9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>Sequence-of-Returns-Risk (SRR) Shield: this engine uses a step function, not a flat percentage. SRR is concentrated in the first years of retirement (the "red zone"), when a bad sequence does the most damage; research supports holding a larger safety anchor through that window, then a smaller one afterward. Each year's actual target -- Red Zone % while Year &lt; Retirement Start Year + Red-Zone-Length, Post-Red-Zone % after -- is computed per-year in the Annual SRR Hurdle Model below and drives the Quarterly Refill Engine's 'Target Safety Anchor Balance (This Year)' column, scaled against that year's simulated wealth path, not a value frozen at Year 1. Row 10 above is only a Year-1 snapshot for quick reference. In this demo, GOOD/POOR below is driven by the Scenario Selector above, not a live account snapshot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="B14" s="22">
+        <f>B3*B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>Sequence-of-Returns-Risk (SRR) Shield: the G Fund target ramps down linearly from the Starting % to the Ending % over the Ramp Length, then holds flat -- SRR is concentrated in the first years of retirement, so the shield is largest when it matters most and eases as that window passes. Each year's actual target is computed per-year in the Annual SRR Hurdle Model below and drives the Quarterly Refill Engine's 'Target Safety Anchor Balance (This Year)' column, scaled against that year's simulated wealth path, not a value frozen at Year 1. The row above is only a Year-1 snapshot for quick reference. In this demo, GOOD/POOR below is driven by the Scenario Selector above, not a live account snapshot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>THE QUARTERLY REFILL ENGINE — PRIMARY OUTPUT: RECOMMENDED TSP TOP-UP TRANSFER</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>Quarterly Outflow (W_q)</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Annual Performance Signal</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>G Fund Balance (Start of Qtr)</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>Recommended Transfer This Quarter</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Actual Transferred (Log It Here)</t>
         </is>
       </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>G Fund Balance (End of Qtr, Projected)</t>
         </is>
       </c>
-      <c r="I14" s="10" t="inlineStr">
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>Target Safety Anchor Balance (This Year)</t>
         </is>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="28" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B15" s="29" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-      <c r="C15" s="30">
-        <f>SUM('Variables_And_Log'!F3:H3)</f>
-        <v/>
-      </c>
-      <c r="D15" s="31">
-        <f>G59</f>
-        <v/>
-      </c>
-      <c r="E15" s="30">
-        <f>'Account_Tracker'!$C$2</f>
-        <v/>
-      </c>
-      <c r="F15" s="32">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D15)),MAX(0,I15-E15),0)</f>
-        <v/>
-      </c>
-      <c r="G15" s="33" t="n"/>
-      <c r="H15" s="30">
-        <f>MAX(0,E15-C15+IF(G15="",F15,G15))</f>
-        <v/>
-      </c>
-      <c r="I15" s="30">
-        <f>H59*D59</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B16" s="20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="C16" s="16">
-        <f>SUM('Variables_And_Log'!I3:K3)</f>
-        <v/>
-      </c>
-      <c r="D16" s="34">
-        <f>G59</f>
-        <v/>
-      </c>
-      <c r="E16" s="16">
-        <f>H15</f>
-        <v/>
-      </c>
-      <c r="F16" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D16)),MAX(0,I16-E16),0)</f>
-        <v/>
-      </c>
-      <c r="G16" s="17" t="n"/>
-      <c r="H16" s="16">
-        <f>MAX(0,E16-C16+IF(G16="",F16,G16))</f>
-        <v/>
-      </c>
-      <c r="I16" s="16">
-        <f>H59*D59</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B17" s="20" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="C17" s="16">
-        <f>SUM('Variables_And_Log'!L3:N3)</f>
-        <v/>
-      </c>
-      <c r="D17" s="34">
-        <f>G59</f>
-        <v/>
-      </c>
-      <c r="E17" s="16">
-        <f>H16</f>
-        <v/>
-      </c>
-      <c r="F17" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D17)),MAX(0,I17-E17),0)</f>
-        <v/>
-      </c>
-      <c r="G17" s="17" t="n"/>
-      <c r="H17" s="16">
-        <f>MAX(0,E17-C17+IF(G17="",F17,G17))</f>
-        <v/>
-      </c>
-      <c r="I17" s="16">
-        <f>H59*D59</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B18" s="20" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="C18" s="16">
-        <f>SUM('Variables_And_Log'!O3:Q3)</f>
-        <v/>
-      </c>
-      <c r="D18" s="34">
-        <f>G59</f>
-        <v/>
-      </c>
-      <c r="E18" s="16">
-        <f>H17</f>
-        <v/>
-      </c>
-      <c r="F18" s="22">
-        <f>IF(ISNUMBER(SEARCH("GOOD",D18)),MAX(0,I18-E18),0)</f>
-        <v/>
-      </c>
-      <c r="G18" s="17" t="n"/>
-      <c r="H18" s="16">
-        <f>MAX(0,E18-C18+IF(G18="",F18,G18))</f>
-        <v/>
-      </c>
-      <c r="I18" s="16">
-        <f>H59*D59</f>
-        <v/>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="28" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B19" s="29" t="inlineStr">
         <is>
@@ -2368,15 +2478,15 @@
         </is>
       </c>
       <c r="C19" s="30">
-        <f>SUM('Variables_And_Log'!F4:H4)</f>
+        <f>SUM('Variables_And_Log'!F3:H3)</f>
         <v/>
       </c>
       <c r="D19" s="31">
-        <f>G60</f>
+        <f>G63</f>
         <v/>
       </c>
       <c r="E19" s="30">
-        <f>H18</f>
+        <f>'Account_Tracker'!$C$2</f>
         <v/>
       </c>
       <c r="F19" s="32">
@@ -2389,13 +2499,13 @@
         <v/>
       </c>
       <c r="I19" s="30">
-        <f>H60*D60</f>
+        <f>H63*D63</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="13" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
@@ -2403,11 +2513,11 @@
         </is>
       </c>
       <c r="C20" s="16">
-        <f>SUM('Variables_And_Log'!I4:K4)</f>
+        <f>SUM('Variables_And_Log'!I3:K3)</f>
         <v/>
       </c>
       <c r="D20" s="34">
-        <f>G60</f>
+        <f>G63</f>
         <v/>
       </c>
       <c r="E20" s="16">
@@ -2424,13 +2534,13 @@
         <v/>
       </c>
       <c r="I20" s="16">
-        <f>H60*D60</f>
+        <f>H63*D63</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="13" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
@@ -2438,11 +2548,11 @@
         </is>
       </c>
       <c r="C21" s="16">
-        <f>SUM('Variables_And_Log'!L4:N4)</f>
+        <f>SUM('Variables_And_Log'!L3:N3)</f>
         <v/>
       </c>
       <c r="D21" s="34">
-        <f>G60</f>
+        <f>G63</f>
         <v/>
       </c>
       <c r="E21" s="16">
@@ -2459,13 +2569,13 @@
         <v/>
       </c>
       <c r="I21" s="16">
-        <f>H60*D60</f>
+        <f>H63*D63</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="13" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="B22" s="20" t="inlineStr">
         <is>
@@ -2473,11 +2583,11 @@
         </is>
       </c>
       <c r="C22" s="16">
-        <f>SUM('Variables_And_Log'!O4:Q4)</f>
+        <f>SUM('Variables_And_Log'!O3:Q3)</f>
         <v/>
       </c>
       <c r="D22" s="34">
-        <f>G60</f>
+        <f>G63</f>
         <v/>
       </c>
       <c r="E22" s="16">
@@ -2494,13 +2604,13 @@
         <v/>
       </c>
       <c r="I22" s="16">
-        <f>H60*D60</f>
+        <f>H63*D63</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="28" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B23" s="29" t="inlineStr">
         <is>
@@ -2508,11 +2618,11 @@
         </is>
       </c>
       <c r="C23" s="30">
-        <f>SUM('Variables_And_Log'!F5:H5)</f>
+        <f>SUM('Variables_And_Log'!F4:H4)</f>
         <v/>
       </c>
       <c r="D23" s="31">
-        <f>G61</f>
+        <f>G64</f>
         <v/>
       </c>
       <c r="E23" s="30">
@@ -2529,13 +2639,13 @@
         <v/>
       </c>
       <c r="I23" s="30">
-        <f>H61*D61</f>
+        <f>H64*D64</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="13" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B24" s="20" t="inlineStr">
         <is>
@@ -2543,11 +2653,11 @@
         </is>
       </c>
       <c r="C24" s="16">
-        <f>SUM('Variables_And_Log'!I5:K5)</f>
+        <f>SUM('Variables_And_Log'!I4:K4)</f>
         <v/>
       </c>
       <c r="D24" s="34">
-        <f>G61</f>
+        <f>G64</f>
         <v/>
       </c>
       <c r="E24" s="16">
@@ -2564,13 +2674,13 @@
         <v/>
       </c>
       <c r="I24" s="16">
-        <f>H61*D61</f>
+        <f>H64*D64</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="13" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B25" s="20" t="inlineStr">
         <is>
@@ -2578,11 +2688,11 @@
         </is>
       </c>
       <c r="C25" s="16">
-        <f>SUM('Variables_And_Log'!L5:N5)</f>
+        <f>SUM('Variables_And_Log'!L4:N4)</f>
         <v/>
       </c>
       <c r="D25" s="34">
-        <f>G61</f>
+        <f>G64</f>
         <v/>
       </c>
       <c r="E25" s="16">
@@ -2599,13 +2709,13 @@
         <v/>
       </c>
       <c r="I25" s="16">
-        <f>H61*D61</f>
+        <f>H64*D64</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="13" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="B26" s="20" t="inlineStr">
         <is>
@@ -2613,11 +2723,11 @@
         </is>
       </c>
       <c r="C26" s="16">
-        <f>SUM('Variables_And_Log'!O5:Q5)</f>
+        <f>SUM('Variables_And_Log'!O4:Q4)</f>
         <v/>
       </c>
       <c r="D26" s="34">
-        <f>G61</f>
+        <f>G64</f>
         <v/>
       </c>
       <c r="E26" s="16">
@@ -2634,13 +2744,13 @@
         <v/>
       </c>
       <c r="I26" s="16">
-        <f>H61*D61</f>
+        <f>H64*D64</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="28" t="n">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B27" s="29" t="inlineStr">
         <is>
@@ -2648,11 +2758,11 @@
         </is>
       </c>
       <c r="C27" s="30">
-        <f>SUM('Variables_And_Log'!F6:H6)</f>
+        <f>SUM('Variables_And_Log'!F5:H5)</f>
         <v/>
       </c>
       <c r="D27" s="31">
-        <f>G62</f>
+        <f>G65</f>
         <v/>
       </c>
       <c r="E27" s="30">
@@ -2669,13 +2779,13 @@
         <v/>
       </c>
       <c r="I27" s="30">
-        <f>H62*D62</f>
+        <f>H65*D65</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="13" t="n">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B28" s="20" t="inlineStr">
         <is>
@@ -2683,11 +2793,11 @@
         </is>
       </c>
       <c r="C28" s="16">
-        <f>SUM('Variables_And_Log'!I6:K6)</f>
+        <f>SUM('Variables_And_Log'!I5:K5)</f>
         <v/>
       </c>
       <c r="D28" s="34">
-        <f>G62</f>
+        <f>G65</f>
         <v/>
       </c>
       <c r="E28" s="16">
@@ -2704,13 +2814,13 @@
         <v/>
       </c>
       <c r="I28" s="16">
-        <f>H62*D62</f>
+        <f>H65*D65</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="13" t="n">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
@@ -2718,11 +2828,11 @@
         </is>
       </c>
       <c r="C29" s="16">
-        <f>SUM('Variables_And_Log'!L6:N6)</f>
+        <f>SUM('Variables_And_Log'!L5:N5)</f>
         <v/>
       </c>
       <c r="D29" s="34">
-        <f>G62</f>
+        <f>G65</f>
         <v/>
       </c>
       <c r="E29" s="16">
@@ -2739,13 +2849,13 @@
         <v/>
       </c>
       <c r="I29" s="16">
-        <f>H62*D62</f>
+        <f>H65*D65</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="13" t="n">
-        <v>2029</v>
+        <v>2028</v>
       </c>
       <c r="B30" s="20" t="inlineStr">
         <is>
@@ -2753,11 +2863,11 @@
         </is>
       </c>
       <c r="C30" s="16">
-        <f>SUM('Variables_And_Log'!O6:Q6)</f>
+        <f>SUM('Variables_And_Log'!O5:Q5)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>G62</f>
+        <f>G65</f>
         <v/>
       </c>
       <c r="E30" s="16">
@@ -2774,13 +2884,13 @@
         <v/>
       </c>
       <c r="I30" s="16">
-        <f>H62*D62</f>
+        <f>H65*D65</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="28" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B31" s="29" t="inlineStr">
         <is>
@@ -2788,11 +2898,11 @@
         </is>
       </c>
       <c r="C31" s="30">
-        <f>SUM('Variables_And_Log'!F7:H7)</f>
+        <f>SUM('Variables_And_Log'!F6:H6)</f>
         <v/>
       </c>
       <c r="D31" s="31">
-        <f>G63</f>
+        <f>G66</f>
         <v/>
       </c>
       <c r="E31" s="30">
@@ -2809,13 +2919,13 @@
         <v/>
       </c>
       <c r="I31" s="30">
-        <f>H63*D63</f>
+        <f>H66*D66</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="13" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B32" s="20" t="inlineStr">
         <is>
@@ -2823,11 +2933,11 @@
         </is>
       </c>
       <c r="C32" s="16">
-        <f>SUM('Variables_And_Log'!I7:K7)</f>
+        <f>SUM('Variables_And_Log'!I6:K6)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>G63</f>
+        <f>G66</f>
         <v/>
       </c>
       <c r="E32" s="16">
@@ -2844,13 +2954,13 @@
         <v/>
       </c>
       <c r="I32" s="16">
-        <f>H63*D63</f>
+        <f>H66*D66</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="13" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B33" s="20" t="inlineStr">
         <is>
@@ -2858,11 +2968,11 @@
         </is>
       </c>
       <c r="C33" s="16">
-        <f>SUM('Variables_And_Log'!L7:N7)</f>
+        <f>SUM('Variables_And_Log'!L6:N6)</f>
         <v/>
       </c>
       <c r="D33" s="34">
-        <f>G63</f>
+        <f>G66</f>
         <v/>
       </c>
       <c r="E33" s="16">
@@ -2879,13 +2989,13 @@
         <v/>
       </c>
       <c r="I33" s="16">
-        <f>H63*D63</f>
+        <f>H66*D66</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="13" t="n">
-        <v>2030</v>
+        <v>2029</v>
       </c>
       <c r="B34" s="20" t="inlineStr">
         <is>
@@ -2893,11 +3003,11 @@
         </is>
       </c>
       <c r="C34" s="16">
-        <f>SUM('Variables_And_Log'!O7:Q7)</f>
+        <f>SUM('Variables_And_Log'!O6:Q6)</f>
         <v/>
       </c>
       <c r="D34" s="34">
-        <f>G63</f>
+        <f>G66</f>
         <v/>
       </c>
       <c r="E34" s="16">
@@ -2914,13 +3024,13 @@
         <v/>
       </c>
       <c r="I34" s="16">
-        <f>H63*D63</f>
+        <f>H66*D66</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="28" t="n">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B35" s="29" t="inlineStr">
         <is>
@@ -2928,11 +3038,11 @@
         </is>
       </c>
       <c r="C35" s="30">
-        <f>SUM('Variables_And_Log'!F8:H8)</f>
+        <f>SUM('Variables_And_Log'!F7:H7)</f>
         <v/>
       </c>
       <c r="D35" s="31">
-        <f>G64</f>
+        <f>G67</f>
         <v/>
       </c>
       <c r="E35" s="30">
@@ -2949,13 +3059,13 @@
         <v/>
       </c>
       <c r="I35" s="30">
-        <f>H64*D64</f>
+        <f>H67*D67</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="13" t="n">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B36" s="20" t="inlineStr">
         <is>
@@ -2963,11 +3073,11 @@
         </is>
       </c>
       <c r="C36" s="16">
-        <f>SUM('Variables_And_Log'!I8:K8)</f>
+        <f>SUM('Variables_And_Log'!I7:K7)</f>
         <v/>
       </c>
       <c r="D36" s="34">
-        <f>G64</f>
+        <f>G67</f>
         <v/>
       </c>
       <c r="E36" s="16">
@@ -2984,13 +3094,13 @@
         <v/>
       </c>
       <c r="I36" s="16">
-        <f>H64*D64</f>
+        <f>H67*D67</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="13" t="n">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B37" s="20" t="inlineStr">
         <is>
@@ -2998,11 +3108,11 @@
         </is>
       </c>
       <c r="C37" s="16">
-        <f>SUM('Variables_And_Log'!L8:N8)</f>
+        <f>SUM('Variables_And_Log'!L7:N7)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>G64</f>
+        <f>G67</f>
         <v/>
       </c>
       <c r="E37" s="16">
@@ -3019,13 +3129,13 @@
         <v/>
       </c>
       <c r="I37" s="16">
-        <f>H64*D64</f>
+        <f>H67*D67</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="13" t="n">
-        <v>2031</v>
+        <v>2030</v>
       </c>
       <c r="B38" s="20" t="inlineStr">
         <is>
@@ -3033,11 +3143,11 @@
         </is>
       </c>
       <c r="C38" s="16">
-        <f>SUM('Variables_And_Log'!O8:Q8)</f>
+        <f>SUM('Variables_And_Log'!O7:Q7)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>G64</f>
+        <f>G67</f>
         <v/>
       </c>
       <c r="E38" s="16">
@@ -3054,13 +3164,13 @@
         <v/>
       </c>
       <c r="I38" s="16">
-        <f>H64*D64</f>
+        <f>H67*D67</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="28" t="n">
-        <v>2032</v>
+        <v>2031</v>
       </c>
       <c r="B39" s="29" t="inlineStr">
         <is>
@@ -3068,11 +3178,11 @@
         </is>
       </c>
       <c r="C39" s="30">
-        <f>SUM('Variables_And_Log'!F9:H9)</f>
+        <f>SUM('Variables_And_Log'!F8:H8)</f>
         <v/>
       </c>
       <c r="D39" s="31">
-        <f>G65</f>
+        <f>G68</f>
         <v/>
       </c>
       <c r="E39" s="30">
@@ -3089,13 +3199,13 @@
         <v/>
       </c>
       <c r="I39" s="30">
-        <f>H65*D65</f>
+        <f>H68*D68</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="13" t="n">
-        <v>2032</v>
+        <v>2031</v>
       </c>
       <c r="B40" s="20" t="inlineStr">
         <is>
@@ -3103,11 +3213,11 @@
         </is>
       </c>
       <c r="C40" s="16">
-        <f>SUM('Variables_And_Log'!I9:K9)</f>
+        <f>SUM('Variables_And_Log'!I8:K8)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>G65</f>
+        <f>G68</f>
         <v/>
       </c>
       <c r="E40" s="16">
@@ -3124,13 +3234,13 @@
         <v/>
       </c>
       <c r="I40" s="16">
-        <f>H65*D65</f>
+        <f>H68*D68</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="13" t="n">
-        <v>2032</v>
+        <v>2031</v>
       </c>
       <c r="B41" s="20" t="inlineStr">
         <is>
@@ -3138,11 +3248,11 @@
         </is>
       </c>
       <c r="C41" s="16">
-        <f>SUM('Variables_And_Log'!L9:N9)</f>
+        <f>SUM('Variables_And_Log'!L8:N8)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>G65</f>
+        <f>G68</f>
         <v/>
       </c>
       <c r="E41" s="16">
@@ -3159,13 +3269,13 @@
         <v/>
       </c>
       <c r="I41" s="16">
-        <f>H65*D65</f>
+        <f>H68*D68</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="13" t="n">
-        <v>2032</v>
+        <v>2031</v>
       </c>
       <c r="B42" s="20" t="inlineStr">
         <is>
@@ -3173,11 +3283,11 @@
         </is>
       </c>
       <c r="C42" s="16">
-        <f>SUM('Variables_And_Log'!O9:Q9)</f>
+        <f>SUM('Variables_And_Log'!O8:Q8)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>G65</f>
+        <f>G68</f>
         <v/>
       </c>
       <c r="E42" s="16">
@@ -3194,13 +3304,13 @@
         <v/>
       </c>
       <c r="I42" s="16">
-        <f>H65*D65</f>
+        <f>H68*D68</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="28" t="n">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="B43" s="29" t="inlineStr">
         <is>
@@ -3208,11 +3318,11 @@
         </is>
       </c>
       <c r="C43" s="30">
-        <f>SUM('Variables_And_Log'!F10:H10)</f>
+        <f>SUM('Variables_And_Log'!F9:H9)</f>
         <v/>
       </c>
       <c r="D43" s="31">
-        <f>G66</f>
+        <f>G69</f>
         <v/>
       </c>
       <c r="E43" s="30">
@@ -3229,13 +3339,13 @@
         <v/>
       </c>
       <c r="I43" s="30">
-        <f>H66*D66</f>
+        <f>H69*D69</f>
         <v/>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="13" t="n">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="B44" s="20" t="inlineStr">
         <is>
@@ -3243,11 +3353,11 @@
         </is>
       </c>
       <c r="C44" s="16">
-        <f>SUM('Variables_And_Log'!I10:K10)</f>
+        <f>SUM('Variables_And_Log'!I9:K9)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>G66</f>
+        <f>G69</f>
         <v/>
       </c>
       <c r="E44" s="16">
@@ -3264,13 +3374,13 @@
         <v/>
       </c>
       <c r="I44" s="16">
-        <f>H66*D66</f>
+        <f>H69*D69</f>
         <v/>
       </c>
     </row>
     <row r="45" ht="28" customHeight="1">
       <c r="A45" s="13" t="n">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="B45" s="20" t="inlineStr">
         <is>
@@ -3278,11 +3388,11 @@
         </is>
       </c>
       <c r="C45" s="16">
-        <f>SUM('Variables_And_Log'!L10:N10)</f>
+        <f>SUM('Variables_And_Log'!L9:N9)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>G66</f>
+        <f>G69</f>
         <v/>
       </c>
       <c r="E45" s="16">
@@ -3299,13 +3409,13 @@
         <v/>
       </c>
       <c r="I45" s="16">
-        <f>H66*D66</f>
+        <f>H69*D69</f>
         <v/>
       </c>
     </row>
     <row r="46" ht="28" customHeight="1">
       <c r="A46" s="13" t="n">
-        <v>2033</v>
+        <v>2032</v>
       </c>
       <c r="B46" s="20" t="inlineStr">
         <is>
@@ -3313,11 +3423,11 @@
         </is>
       </c>
       <c r="C46" s="16">
-        <f>SUM('Variables_And_Log'!O10:Q10)</f>
+        <f>SUM('Variables_And_Log'!O9:Q9)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>G66</f>
+        <f>G69</f>
         <v/>
       </c>
       <c r="E46" s="16">
@@ -3334,13 +3444,13 @@
         <v/>
       </c>
       <c r="I46" s="16">
-        <f>H66*D66</f>
+        <f>H69*D69</f>
         <v/>
       </c>
     </row>
     <row r="47" ht="28" customHeight="1">
       <c r="A47" s="28" t="n">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="B47" s="29" t="inlineStr">
         <is>
@@ -3348,11 +3458,11 @@
         </is>
       </c>
       <c r="C47" s="30">
-        <f>SUM('Variables_And_Log'!F11:H11)</f>
+        <f>SUM('Variables_And_Log'!F10:H10)</f>
         <v/>
       </c>
       <c r="D47" s="31">
-        <f>G67</f>
+        <f>G70</f>
         <v/>
       </c>
       <c r="E47" s="30">
@@ -3369,13 +3479,13 @@
         <v/>
       </c>
       <c r="I47" s="30">
-        <f>H67*D67</f>
+        <f>H70*D70</f>
         <v/>
       </c>
     </row>
     <row r="48" ht="28" customHeight="1">
       <c r="A48" s="13" t="n">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="B48" s="20" t="inlineStr">
         <is>
@@ -3383,11 +3493,11 @@
         </is>
       </c>
       <c r="C48" s="16">
-        <f>SUM('Variables_And_Log'!I11:K11)</f>
+        <f>SUM('Variables_And_Log'!I10:K10)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>G67</f>
+        <f>G70</f>
         <v/>
       </c>
       <c r="E48" s="16">
@@ -3404,13 +3514,13 @@
         <v/>
       </c>
       <c r="I48" s="16">
-        <f>H67*D67</f>
+        <f>H70*D70</f>
         <v/>
       </c>
     </row>
     <row r="49" ht="28" customHeight="1">
       <c r="A49" s="13" t="n">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="B49" s="20" t="inlineStr">
         <is>
@@ -3418,11 +3528,11 @@
         </is>
       </c>
       <c r="C49" s="16">
-        <f>SUM('Variables_And_Log'!L11:N11)</f>
+        <f>SUM('Variables_And_Log'!L10:N10)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>G67</f>
+        <f>G70</f>
         <v/>
       </c>
       <c r="E49" s="16">
@@ -3439,13 +3549,13 @@
         <v/>
       </c>
       <c r="I49" s="16">
-        <f>H67*D67</f>
+        <f>H70*D70</f>
         <v/>
       </c>
     </row>
     <row r="50" ht="28" customHeight="1">
       <c r="A50" s="13" t="n">
-        <v>2034</v>
+        <v>2033</v>
       </c>
       <c r="B50" s="20" t="inlineStr">
         <is>
@@ -3453,11 +3563,11 @@
         </is>
       </c>
       <c r="C50" s="16">
-        <f>SUM('Variables_And_Log'!O11:Q11)</f>
+        <f>SUM('Variables_And_Log'!O10:Q10)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>G67</f>
+        <f>G70</f>
         <v/>
       </c>
       <c r="E50" s="16">
@@ -3474,13 +3584,13 @@
         <v/>
       </c>
       <c r="I50" s="16">
-        <f>H67*D67</f>
+        <f>H70*D70</f>
         <v/>
       </c>
     </row>
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="28" t="n">
-        <v>2035</v>
+        <v>2034</v>
       </c>
       <c r="B51" s="29" t="inlineStr">
         <is>
@@ -3488,11 +3598,11 @@
         </is>
       </c>
       <c r="C51" s="30">
-        <f>SUM('Variables_And_Log'!F12:H12)</f>
+        <f>SUM('Variables_And_Log'!F11:H11)</f>
         <v/>
       </c>
       <c r="D51" s="31">
-        <f>G68</f>
+        <f>G71</f>
         <v/>
       </c>
       <c r="E51" s="30">
@@ -3509,13 +3619,13 @@
         <v/>
       </c>
       <c r="I51" s="30">
-        <f>H68*D68</f>
+        <f>H71*D71</f>
         <v/>
       </c>
     </row>
     <row r="52" ht="28" customHeight="1">
       <c r="A52" s="13" t="n">
-        <v>2035</v>
+        <v>2034</v>
       </c>
       <c r="B52" s="20" t="inlineStr">
         <is>
@@ -3523,11 +3633,11 @@
         </is>
       </c>
       <c r="C52" s="16">
-        <f>SUM('Variables_And_Log'!I12:K12)</f>
+        <f>SUM('Variables_And_Log'!I11:K11)</f>
         <v/>
       </c>
       <c r="D52" s="34">
-        <f>G68</f>
+        <f>G71</f>
         <v/>
       </c>
       <c r="E52" s="16">
@@ -3544,13 +3654,13 @@
         <v/>
       </c>
       <c r="I52" s="16">
-        <f>H68*D68</f>
+        <f>H71*D71</f>
         <v/>
       </c>
     </row>
     <row r="53" ht="28" customHeight="1">
       <c r="A53" s="13" t="n">
-        <v>2035</v>
+        <v>2034</v>
       </c>
       <c r="B53" s="20" t="inlineStr">
         <is>
@@ -3558,11 +3668,11 @@
         </is>
       </c>
       <c r="C53" s="16">
-        <f>SUM('Variables_And_Log'!L12:N12)</f>
+        <f>SUM('Variables_And_Log'!L11:N11)</f>
         <v/>
       </c>
       <c r="D53" s="34">
-        <f>G68</f>
+        <f>G71</f>
         <v/>
       </c>
       <c r="E53" s="16">
@@ -3579,13 +3689,13 @@
         <v/>
       </c>
       <c r="I53" s="16">
-        <f>H68*D68</f>
+        <f>H71*D71</f>
         <v/>
       </c>
     </row>
     <row r="54" ht="28" customHeight="1">
       <c r="A54" s="13" t="n">
-        <v>2035</v>
+        <v>2034</v>
       </c>
       <c r="B54" s="20" t="inlineStr">
         <is>
@@ -3593,11 +3703,11 @@
         </is>
       </c>
       <c r="C54" s="16">
-        <f>SUM('Variables_And_Log'!O12:Q12)</f>
+        <f>SUM('Variables_And_Log'!O11:Q11)</f>
         <v/>
       </c>
       <c r="D54" s="34">
-        <f>G68</f>
+        <f>G71</f>
         <v/>
       </c>
       <c r="E54" s="16">
@@ -3614,222 +3724,230 @@
         <v/>
       </c>
       <c r="I54" s="16">
-        <f>H68*D68</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57" ht="20" customHeight="1">
-      <c r="A57" s="2" t="inlineStr">
+        <f>H71*D71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="28" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B55" s="29" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C55" s="30">
+        <f>SUM('Variables_And_Log'!F12:H12)</f>
+        <v/>
+      </c>
+      <c r="D55" s="31">
+        <f>G72</f>
+        <v/>
+      </c>
+      <c r="E55" s="30">
+        <f>H54</f>
+        <v/>
+      </c>
+      <c r="F55" s="32">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D55)),MAX(0,I55-E55),0)</f>
+        <v/>
+      </c>
+      <c r="G55" s="33" t="n"/>
+      <c r="H55" s="30">
+        <f>MAX(0,E55-C55+IF(G55="",F55,G55))</f>
+        <v/>
+      </c>
+      <c r="I55" s="30">
+        <f>H72*D72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="13" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B56" s="20" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C56" s="16">
+        <f>SUM('Variables_And_Log'!I12:K12)</f>
+        <v/>
+      </c>
+      <c r="D56" s="34">
+        <f>G72</f>
+        <v/>
+      </c>
+      <c r="E56" s="16">
+        <f>H55</f>
+        <v/>
+      </c>
+      <c r="F56" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D56)),MAX(0,I56-E56),0)</f>
+        <v/>
+      </c>
+      <c r="G56" s="17" t="n"/>
+      <c r="H56" s="16">
+        <f>MAX(0,E56-C56+IF(G56="",F56,G56))</f>
+        <v/>
+      </c>
+      <c r="I56" s="16">
+        <f>H72*D72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" ht="28" customHeight="1">
+      <c r="A57" s="13" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B57" s="20" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="C57" s="16">
+        <f>SUM('Variables_And_Log'!L12:N12)</f>
+        <v/>
+      </c>
+      <c r="D57" s="34">
+        <f>G72</f>
+        <v/>
+      </c>
+      <c r="E57" s="16">
+        <f>H56</f>
+        <v/>
+      </c>
+      <c r="F57" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D57)),MAX(0,I57-E57),0)</f>
+        <v/>
+      </c>
+      <c r="G57" s="17" t="n"/>
+      <c r="H57" s="16">
+        <f>MAX(0,E57-C57+IF(G57="",F57,G57))</f>
+        <v/>
+      </c>
+      <c r="I57" s="16">
+        <f>H72*D72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="A58" s="13" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B58" s="20" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="C58" s="16">
+        <f>SUM('Variables_And_Log'!O12:Q12)</f>
+        <v/>
+      </c>
+      <c r="D58" s="34">
+        <f>G72</f>
+        <v/>
+      </c>
+      <c r="E58" s="16">
+        <f>H57</f>
+        <v/>
+      </c>
+      <c r="F58" s="22">
+        <f>IF(ISNUMBER(SEARCH("GOOD",D58)),MAX(0,I58-E58),0)</f>
+        <v/>
+      </c>
+      <c r="G58" s="17" t="n"/>
+      <c r="H58" s="16">
+        <f>MAX(0,E58-C58+IF(G58="",F58,G58))</f>
+        <v/>
+      </c>
+      <c r="I58" s="16">
+        <f>H72*D72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>ANNUAL SRR HURDLE MODEL — SIMULATED WEALTH VS. HURDLE (GATES THE QUARTERLY REFILL ABOVE)</t>
         </is>
       </c>
-      <c r="B57" s="2" t="n"/>
-      <c r="C57" s="2" t="n"/>
-      <c r="D57" s="2" t="n"/>
-      <c r="E57" s="2" t="n"/>
-      <c r="F57" s="2" t="n"/>
-      <c r="G57" s="2" t="n"/>
-      <c r="H57" s="2" t="n"/>
-    </row>
-    <row r="58" ht="40" customHeight="1">
-      <c r="A58" s="10" t="inlineStr">
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+      <c r="E61" s="2" t="n"/>
+      <c r="F61" s="2" t="n"/>
+      <c r="G61" s="2" t="n"/>
+      <c r="H61" s="2" t="n"/>
+    </row>
+    <row r="62" ht="40" customHeight="1">
+      <c r="A62" s="10" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B58" s="10" t="inlineStr">
+      <c r="B62" s="10" t="inlineStr">
         <is>
           <t>Total Annual Hurdle Rate</t>
         </is>
       </c>
-      <c r="C58" s="10" t="inlineStr">
+      <c r="C62" s="10" t="inlineStr">
         <is>
           <t>Annual Outflows (W_t)</t>
         </is>
       </c>
-      <c r="D58" s="10" t="inlineStr">
+      <c r="D62" s="10" t="inlineStr">
         <is>
           <t>Simulated Target Portfolio (P_track)</t>
         </is>
       </c>
-      <c r="E58" s="10" t="inlineStr">
+      <c r="E62" s="10" t="inlineStr">
         <is>
           <t>Scenario Return (Selected, This Year)</t>
         </is>
       </c>
-      <c r="F58" s="10" t="inlineStr">
+      <c r="F62" s="10" t="inlineStr">
         <is>
           <t>Simulated Actual Household Wealth (This Year)</t>
         </is>
       </c>
-      <c r="G58" s="10" t="inlineStr">
+      <c r="G62" s="10" t="inlineStr">
         <is>
           <t>Performance Logic Trigger</t>
         </is>
       </c>
-      <c r="H58" s="10" t="inlineStr">
+      <c r="H62" s="10" t="inlineStr">
         <is>
           <t>Safety Anchor % (This Year)</t>
         </is>
-      </c>
-    </row>
-    <row r="59" ht="28" customHeight="1">
-      <c r="A59" s="13" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B59" s="15">
-        <f>'Variables_And_Log'!D3</f>
-        <v/>
-      </c>
-      <c r="C59" s="16">
-        <f>'Variables_And_Log'!E3</f>
-        <v/>
-      </c>
-      <c r="D59" s="16">
-        <f>ROUND(($B$3*B59)-C59,2)</f>
-        <v/>
-      </c>
-      <c r="E59" s="15">
-        <f>'Variables_And_Log'!U3</f>
-        <v/>
-      </c>
-      <c r="F59" s="22">
-        <f>ROUND(($B$3*(1+E59))-C59,2)</f>
-        <v/>
-      </c>
-      <c r="G59" s="34">
-        <f>IF(F59&gt;=D59,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
-        <v/>
-      </c>
-      <c r="H59" s="15">
-        <f>IF(A59-$B$4&lt;$B$6,$B$7,$B$8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="28" customHeight="1">
-      <c r="A60" s="13" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B60" s="15">
-        <f>'Variables_And_Log'!D4</f>
-        <v/>
-      </c>
-      <c r="C60" s="16">
-        <f>'Variables_And_Log'!E4</f>
-        <v/>
-      </c>
-      <c r="D60" s="16">
-        <f>ROUND((D59*B60)-C60,2)</f>
-        <v/>
-      </c>
-      <c r="E60" s="15">
-        <f>'Variables_And_Log'!U4</f>
-        <v/>
-      </c>
-      <c r="F60" s="22">
-        <f>ROUND((F59*(1+E60))-C60,2)</f>
-        <v/>
-      </c>
-      <c r="G60" s="34">
-        <f>IF(F60&gt;=D60,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
-        <v/>
-      </c>
-      <c r="H60" s="15">
-        <f>IF(A60-$B$4&lt;$B$6,$B$7,$B$8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" ht="28" customHeight="1">
-      <c r="A61" s="13" t="n">
-        <v>2028</v>
-      </c>
-      <c r="B61" s="15">
-        <f>'Variables_And_Log'!D5</f>
-        <v/>
-      </c>
-      <c r="C61" s="16">
-        <f>'Variables_And_Log'!E5</f>
-        <v/>
-      </c>
-      <c r="D61" s="16">
-        <f>ROUND((D60*B61)-C61,2)</f>
-        <v/>
-      </c>
-      <c r="E61" s="15">
-        <f>'Variables_And_Log'!U5</f>
-        <v/>
-      </c>
-      <c r="F61" s="22">
-        <f>ROUND((F60*(1+E61))-C61,2)</f>
-        <v/>
-      </c>
-      <c r="G61" s="34">
-        <f>IF(F61&gt;=D61,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
-        <v/>
-      </c>
-      <c r="H61" s="15">
-        <f>IF(A61-$B$4&lt;$B$6,$B$7,$B$8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" ht="28" customHeight="1">
-      <c r="A62" s="13" t="n">
-        <v>2029</v>
-      </c>
-      <c r="B62" s="15">
-        <f>'Variables_And_Log'!D6</f>
-        <v/>
-      </c>
-      <c r="C62" s="16">
-        <f>'Variables_And_Log'!E6</f>
-        <v/>
-      </c>
-      <c r="D62" s="16">
-        <f>ROUND((D61*B62)-C62,2)</f>
-        <v/>
-      </c>
-      <c r="E62" s="15">
-        <f>'Variables_And_Log'!U6</f>
-        <v/>
-      </c>
-      <c r="F62" s="22">
-        <f>ROUND((F61*(1+E62))-C62,2)</f>
-        <v/>
-      </c>
-      <c r="G62" s="34">
-        <f>IF(F62&gt;=D62,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
-        <v/>
-      </c>
-      <c r="H62" s="15">
-        <f>IF(A62-$B$4&lt;$B$6,$B$7,$B$8)</f>
-        <v/>
       </c>
     </row>
     <row r="63" ht="28" customHeight="1">
       <c r="A63" s="13" t="n">
-        <v>2030</v>
+        <v>2026</v>
       </c>
       <c r="B63" s="15">
-        <f>'Variables_And_Log'!D7</f>
+        <f>'Variables_And_Log'!D3</f>
         <v/>
       </c>
       <c r="C63" s="16">
-        <f>'Variables_And_Log'!E7</f>
+        <f>'Variables_And_Log'!E3</f>
         <v/>
       </c>
       <c r="D63" s="16">
-        <f>ROUND((D62*B63)-C63,2)</f>
+        <f>ROUND(($B$3*B63)-C63,2)</f>
         <v/>
       </c>
       <c r="E63" s="15">
-        <f>'Variables_And_Log'!U7</f>
+        <f>'Variables_And_Log'!U3</f>
         <v/>
       </c>
       <c r="F63" s="22">
-        <f>ROUND((F62*(1+E63))-C63,2)</f>
+        <f>ROUND(($B$3*(1+E63))-C63,2)</f>
         <v/>
       </c>
       <c r="G63" s="34">
@@ -3837,20 +3955,20 @@
         <v/>
       </c>
       <c r="H63" s="15">
-        <f>IF(A63-$B$4&lt;$B$6,$B$7,$B$8)</f>
+        <f>IF(A63-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(A63-$D$7)/$D$9)</f>
         <v/>
       </c>
     </row>
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="13" t="n">
-        <v>2031</v>
+        <v>2027</v>
       </c>
       <c r="B64" s="15">
-        <f>'Variables_And_Log'!D8</f>
+        <f>'Variables_And_Log'!D4</f>
         <v/>
       </c>
       <c r="C64" s="16">
-        <f>'Variables_And_Log'!E8</f>
+        <f>'Variables_And_Log'!E4</f>
         <v/>
       </c>
       <c r="D64" s="16">
@@ -3858,7 +3976,7 @@
         <v/>
       </c>
       <c r="E64" s="15">
-        <f>'Variables_And_Log'!U8</f>
+        <f>'Variables_And_Log'!U4</f>
         <v/>
       </c>
       <c r="F64" s="22">
@@ -3870,20 +3988,20 @@
         <v/>
       </c>
       <c r="H64" s="15">
-        <f>IF(A64-$B$4&lt;$B$6,$B$7,$B$8)</f>
+        <f>IF(A64-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(A64-$D$7)/$D$9)</f>
         <v/>
       </c>
     </row>
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="13" t="n">
-        <v>2032</v>
+        <v>2028</v>
       </c>
       <c r="B65" s="15">
-        <f>'Variables_And_Log'!D9</f>
+        <f>'Variables_And_Log'!D5</f>
         <v/>
       </c>
       <c r="C65" s="16">
-        <f>'Variables_And_Log'!E9</f>
+        <f>'Variables_And_Log'!E5</f>
         <v/>
       </c>
       <c r="D65" s="16">
@@ -3891,7 +4009,7 @@
         <v/>
       </c>
       <c r="E65" s="15">
-        <f>'Variables_And_Log'!U9</f>
+        <f>'Variables_And_Log'!U5</f>
         <v/>
       </c>
       <c r="F65" s="22">
@@ -3903,20 +4021,20 @@
         <v/>
       </c>
       <c r="H65" s="15">
-        <f>IF(A65-$B$4&lt;$B$6,$B$7,$B$8)</f>
+        <f>IF(A65-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(A65-$D$7)/$D$9)</f>
         <v/>
       </c>
     </row>
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="13" t="n">
-        <v>2033</v>
+        <v>2029</v>
       </c>
       <c r="B66" s="15">
-        <f>'Variables_And_Log'!D10</f>
+        <f>'Variables_And_Log'!D6</f>
         <v/>
       </c>
       <c r="C66" s="16">
-        <f>'Variables_And_Log'!E10</f>
+        <f>'Variables_And_Log'!E6</f>
         <v/>
       </c>
       <c r="D66" s="16">
@@ -3924,7 +4042,7 @@
         <v/>
       </c>
       <c r="E66" s="15">
-        <f>'Variables_And_Log'!U10</f>
+        <f>'Variables_And_Log'!U6</f>
         <v/>
       </c>
       <c r="F66" s="22">
@@ -3936,20 +4054,20 @@
         <v/>
       </c>
       <c r="H66" s="15">
-        <f>IF(A66-$B$4&lt;$B$6,$B$7,$B$8)</f>
+        <f>IF(A66-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(A66-$D$7)/$D$9)</f>
         <v/>
       </c>
     </row>
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="13" t="n">
-        <v>2034</v>
+        <v>2030</v>
       </c>
       <c r="B67" s="15">
-        <f>'Variables_And_Log'!D11</f>
+        <f>'Variables_And_Log'!D7</f>
         <v/>
       </c>
       <c r="C67" s="16">
-        <f>'Variables_And_Log'!E11</f>
+        <f>'Variables_And_Log'!E7</f>
         <v/>
       </c>
       <c r="D67" s="16">
@@ -3957,7 +4075,7 @@
         <v/>
       </c>
       <c r="E67" s="15">
-        <f>'Variables_And_Log'!U11</f>
+        <f>'Variables_And_Log'!U7</f>
         <v/>
       </c>
       <c r="F67" s="22">
@@ -3969,20 +4087,20 @@
         <v/>
       </c>
       <c r="H67" s="15">
-        <f>IF(A67-$B$4&lt;$B$6,$B$7,$B$8)</f>
+        <f>IF(A67-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(A67-$D$7)/$D$9)</f>
         <v/>
       </c>
     </row>
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="13" t="n">
-        <v>2035</v>
+        <v>2031</v>
       </c>
       <c r="B68" s="15">
-        <f>'Variables_And_Log'!D12</f>
+        <f>'Variables_And_Log'!D8</f>
         <v/>
       </c>
       <c r="C68" s="16">
-        <f>'Variables_And_Log'!E12</f>
+        <f>'Variables_And_Log'!E8</f>
         <v/>
       </c>
       <c r="D68" s="16">
@@ -3990,7 +4108,7 @@
         <v/>
       </c>
       <c r="E68" s="15">
-        <f>'Variables_And_Log'!U12</f>
+        <f>'Variables_And_Log'!U8</f>
         <v/>
       </c>
       <c r="F68" s="22">
@@ -4002,114 +4120,247 @@
         <v/>
       </c>
       <c r="H68" s="15">
-        <f>IF(A68-$B$4&lt;$B$6,$B$7,$B$8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69"/>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+        <f>IF(A68-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(A68-$D$7)/$D$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" ht="28" customHeight="1">
+      <c r="A69" s="13" t="n">
+        <v>2032</v>
+      </c>
+      <c r="B69" s="15">
+        <f>'Variables_And_Log'!D9</f>
+        <v/>
+      </c>
+      <c r="C69" s="16">
+        <f>'Variables_And_Log'!E9</f>
+        <v/>
+      </c>
+      <c r="D69" s="16">
+        <f>ROUND((D68*B69)-C69,2)</f>
+        <v/>
+      </c>
+      <c r="E69" s="15">
+        <f>'Variables_And_Log'!U9</f>
+        <v/>
+      </c>
+      <c r="F69" s="22">
+        <f>ROUND((F68*(1+E69))-C69,2)</f>
+        <v/>
+      </c>
+      <c r="G69" s="34">
+        <f>IF(F69&gt;=D69,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="H69" s="15">
+        <f>IF(A69-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(A69-$D$7)/$D$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="28" customHeight="1">
+      <c r="A70" s="13" t="n">
+        <v>2033</v>
+      </c>
+      <c r="B70" s="15">
+        <f>'Variables_And_Log'!D10</f>
+        <v/>
+      </c>
+      <c r="C70" s="16">
+        <f>'Variables_And_Log'!E10</f>
+        <v/>
+      </c>
+      <c r="D70" s="16">
+        <f>ROUND((D69*B70)-C70,2)</f>
+        <v/>
+      </c>
+      <c r="E70" s="15">
+        <f>'Variables_And_Log'!U10</f>
+        <v/>
+      </c>
+      <c r="F70" s="22">
+        <f>ROUND((F69*(1+E70))-C70,2)</f>
+        <v/>
+      </c>
+      <c r="G70" s="34">
+        <f>IF(F70&gt;=D70,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="H70" s="15">
+        <f>IF(A70-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(A70-$D$7)/$D$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="28" customHeight="1">
+      <c r="A71" s="13" t="n">
+        <v>2034</v>
+      </c>
+      <c r="B71" s="15">
+        <f>'Variables_And_Log'!D11</f>
+        <v/>
+      </c>
+      <c r="C71" s="16">
+        <f>'Variables_And_Log'!E11</f>
+        <v/>
+      </c>
+      <c r="D71" s="16">
+        <f>ROUND((D70*B71)-C71,2)</f>
+        <v/>
+      </c>
+      <c r="E71" s="15">
+        <f>'Variables_And_Log'!U11</f>
+        <v/>
+      </c>
+      <c r="F71" s="22">
+        <f>ROUND((F70*(1+E71))-C71,2)</f>
+        <v/>
+      </c>
+      <c r="G71" s="34">
+        <f>IF(F71&gt;=D71,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="H71" s="15">
+        <f>IF(A71-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(A71-$D$7)/$D$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" ht="28" customHeight="1">
+      <c r="A72" s="13" t="n">
+        <v>2035</v>
+      </c>
+      <c r="B72" s="15">
+        <f>'Variables_And_Log'!D12</f>
+        <v/>
+      </c>
+      <c r="C72" s="16">
+        <f>'Variables_And_Log'!E12</f>
+        <v/>
+      </c>
+      <c r="D72" s="16">
+        <f>ROUND((D71*B72)-C72,2)</f>
+        <v/>
+      </c>
+      <c r="E72" s="15">
+        <f>'Variables_And_Log'!U12</f>
+        <v/>
+      </c>
+      <c r="F72" s="22">
+        <f>ROUND((F71*(1+E72))-C72,2)</f>
+        <v/>
+      </c>
+      <c r="G72" s="34">
+        <f>IF(F72&gt;=D72,"✅ GOOD: Execute T2065 Rebalance &amp; Rollover to TSP","⚠️ POOR: Freeze Equities. Draw Down G Fund")</f>
+        <v/>
+      </c>
+      <c r="H72" s="15">
+        <f>IF(A72-$D$7&gt;=$D$9,$D$11,$D$10+($D$11-$D$10)*(A72-$D$7)/$D$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73"/>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t>EXTRA CAPACITY INDICATORS</t>
         </is>
       </c>
-      <c r="B70" s="2" t="n"/>
-      <c r="C70" s="2" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="24" t="inlineStr">
+      <c r="B74" s="2" t="n"/>
+      <c r="C74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="24" t="inlineStr">
         <is>
           <t>Your Pre-Tax Rollover Conduit Capacity</t>
         </is>
       </c>
-      <c r="B71" s="16">
+      <c r="B75" s="16">
         <f>'Account_Tracker'!$C$3</f>
         <v/>
       </c>
-      <c r="C71" s="21">
-        <f>IF(B71&gt;0,"Conduit Open","Conduit Closed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72"/>
-    <row r="73">
-      <c r="A73" s="24" t="inlineStr">
+      <c r="C75" s="21">
+        <f>IF(B75&gt;0,"Conduit Open","Conduit Closed")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76"/>
+    <row r="77">
+      <c r="A77" s="24" t="inlineStr">
         <is>
           <t>TSP Cash Buffer Runway (Months)</t>
         </is>
       </c>
-      <c r="B73" s="35">
+      <c r="B77" s="35">
         <f>IFERROR('Account_Tracker'!$C$2/AVERAGE('Variables_And_Log'!$F$3:$Q$3),"Log Monthly Payments to Calculate")</f>
         <v/>
       </c>
-      <c r="C73" s="21">
-        <f>IF(ISNUMBER(B73),IF(B73&gt;36,"Safe: 3+ Year Volatility Shield","Caution: Shield Shrinking"),"Awaiting Payment Data")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="19" t="inlineStr">
+      <c r="C77" s="21">
+        <f>IF(ISNUMBER(B77),IF(B77&gt;36,"Safe: 3+ Year Volatility Shield","Caution: Shield Shrinking"),"Awaiting Payment Data")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="19" t="inlineStr">
         <is>
           <t>(Runway uses the average of 2026's monthly TSP payments, and the G Fund's Year-1 starting balance -- it does not reflect the quarter-by-quarter projection above.)</t>
         </is>
       </c>
     </row>
-    <row r="75"/>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
+    <row r="79"/>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>EMERGENCY LIQUIDITY PROTOCOL — NEXT-DOLLAR PRIORITY ENGINE</t>
         </is>
       </c>
-      <c r="B76" s="2" t="n"/>
-      <c r="C76" s="2" t="n"/>
-      <c r="D76" s="2" t="n"/>
-      <c r="E76" s="2" t="n"/>
-    </row>
-    <row r="77" ht="60" customHeight="1">
-      <c r="A77" s="24" t="inlineStr">
+      <c r="B80" s="2" t="n"/>
+      <c r="C80" s="2" t="n"/>
+      <c r="D80" s="2" t="n"/>
+      <c r="E80" s="2" t="n"/>
+    </row>
+    <row r="81" ht="60" customHeight="1">
+      <c r="A81" s="24" t="inlineStr">
         <is>
           <t>Next-Dollar Liquidity Priority</t>
         </is>
       </c>
-      <c r="B77" s="36">
+      <c r="B81" s="36">
         <f>IF('Account_Tracker'!$C$2&gt;0,"🛡️ SHIELD ACTIVE: Continue automated monthly draws directly from the TSP G Fund. Your equity engines are fully insulated from sequence-of-returns risk.",IF(AND('Account_Tracker'!$C$2=0,'Account_Tracker'!$C$8&gt;0),"⚠️ SHIELD BROKEN: TSP G Fund is exhausted. IMMEDIATELY divert monthly checking draws to your Merrill Edge Cash Buffer. This buys next-day liquidity via Bank of America without forced retirement asset sales.",IF(AND('Account_Tracker'!$C$2=0,'Account_Tracker'!$C$8=0,'Account_Tracker'!$C$6&gt;0),"🚨 EMERGENCY LIQUIDATION - STAGE 1: G Fund and Cash Buffers are exhausted. Turn on monthly distributions from Spouse's Current Employer 403b. Their pre-tax employer plan qualifies for the Maryland Pension Exclusion at age 65, making it more tax-efficient than touching your private traditional IRA.","💥 NUCLEAR PROTOCOL - STAGE 2: Absolute liquidity crisis. You are forced to break all shields. Begin selling shares of the 2065 Target Date Funds within your Private Traditional IRAs to fund monthly expenses. Maximize tax withholding at the time of distribution to shield your remaining capital from underpayment penalties.")))</f>
         <v/>
       </c>
-      <c r="C77" s="5" t="n"/>
-      <c r="D77" s="5" t="n"/>
-      <c r="E77" s="5" t="n"/>
-    </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="B78" s="5" t="n"/>
-      <c r="C78" s="5" t="n"/>
-      <c r="D78" s="5" t="n"/>
-      <c r="E78" s="5" t="n"/>
-    </row>
-    <row r="79" ht="20" customHeight="1">
-      <c r="B79" s="5" t="n"/>
-      <c r="C79" s="5" t="n"/>
-      <c r="D79" s="5" t="n"/>
-      <c r="E79" s="5" t="n"/>
-    </row>
-    <row r="80"/>
-    <row r="81">
-      <c r="A81" s="19" t="inlineStr">
+      <c r="C81" s="5" t="n"/>
+      <c r="D81" s="5" t="n"/>
+      <c r="E81" s="5" t="n"/>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="B82" s="5" t="n"/>
+      <c r="C82" s="5" t="n"/>
+      <c r="D82" s="5" t="n"/>
+      <c r="E82" s="5" t="n"/>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="B83" s="5" t="n"/>
+      <c r="C83" s="5" t="n"/>
+      <c r="D83" s="5" t="n"/>
+      <c r="E83" s="5" t="n"/>
+    </row>
+    <row r="84"/>
+    <row r="85">
+      <c r="A85" s="19" t="inlineStr">
         <is>
           <t>Legend: pale-yellow cells are yours to type into (pre-filled here with illustrative example numbers); white cells hold formulas or fixed scenario assumptions -- please don't overwrite them.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="B77:E79"/>
-    <mergeCell ref="A57:H57"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A76:E76"/>
-    <mergeCell ref="A70:C70"/>
+  <mergeCells count="7">
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="B81:E83"/>
+    <mergeCell ref="A74:C74"/>
+    <mergeCell ref="A17:I17"/>
     <mergeCell ref="C1:I1"/>
+    <mergeCell ref="A80:E80"/>
+    <mergeCell ref="A61:H61"/>
   </mergeCells>
-  <conditionalFormatting sqref="B77:B79">
+  <conditionalFormatting sqref="B81:B83">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>'Account_Tracker'!$C$2&gt;0</formula>
     </cfRule>
@@ -4127,4 +4378,41 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SIMULATED WEALTH VS. HURDLE — SELECTED SCENARIO</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+    </row>
+    <row r="3" ht="68" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>This chart reads directly from the Annual SRR Hurdle Model table on The_Refill_Engine -- there is nothing to edit here. It redraws automatically for whichever scenario is selected there: watch Simulated Actual Household Wealth stay under the hurdle (P_track) for the whole Bear run, clear it every year under Bull, and cross back and forth under Choppy.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>